<commit_message>
Enrich MO disability/IME list with verified contacts; add CSV + DDS fix
- Folded researched provider-onboarding contacts (URLs, phones, emails)
  into the Excel; added Provider/join URL, Phone, Email columns.
- Applied corrections: MO DDS under DESE Voc Rehab; IMX now Leidos QTC;
  MATA matanet.org; Legion missourilegion.org; Sterling sterlingmedcorp.com;
  mdexams -> MDSI.
- Corrected DDS reference in outreach packet Template B.
- Added CSV export used to create the Google Sheet copy in Drive.

https://claude.ai/code/session_01UPpefrjLvassqcshMe3M2N
</commit_message>
<xml_diff>
--- a/GFM_Missouri_Disability_IME_List.xlsx
+++ b/GFM_Missouri_Disability_IME_List.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="MO Disability + IME List" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MO Disability + IME List" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -130,16 +130,14 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -507,19 +505,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -550,25 +550,35 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Provider / join URL</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>How to engage (provider / vendor sign-up)</t>
+          <t>Phone</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Email / contact</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>How to apply</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Missouri relevance</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Status / Notes</t>
         </is>
@@ -577,7 +587,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>VA disability — C&amp;P exam TPAs (contract licensed MO physicians to perform Compensation &amp; Pension exams)</t>
+          <t>VA disability — C&amp;P exam TPAs (contract licensed MO physicians to perform Compensation &amp; Pension / disability exams)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n"/>
@@ -589,6 +599,8 @@
       <c r="H2" s="3" t="n"/>
       <c r="I2" s="3" t="n"/>
       <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -596,7 +608,7 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>QTC Medical Services (a Leidos company)</t>
+          <t>QTC Medical Services (Leidos QTC Health Services)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
@@ -616,27 +628,37 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>qtcm.com</t>
+          <t>qtcm.com/providers</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Apply via 'Provider Network' / 'Join our network' page; credentialing required.</t>
+          <t>800-682-9701</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Serves MO veterans; needs in-state examining providers.</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
+          <t>Web form: qtcm.com/contact-us</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Apply via Providers page; active unrestricted MO license; orientation before first exam.</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>Serves MO veterans; needs in-state examiners.</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Top target — verify current provider intake email/phone.</t>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Top target. Note: IMX (#13) now rolls up under Leidos QTC.</t>
         </is>
       </c>
     </row>
@@ -646,7 +668,7 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>VES – Veterans Evaluation Services (a Maximus company)</t>
+          <t>VES – Veterans Evaluation Services (Maximus)</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -656,7 +678,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Major VA disability exam contractor; builds nationwide examiner network.</t>
+          <t>Major VA disability exam contractor building a nationwide examiner network.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -666,27 +688,37 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>vesservices.com</t>
+          <t>ves.com/providers</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>'Providers' &gt; join network; submit CV, licenses, board certs.</t>
+          <t>877-637-8387</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Contracts MO-licensed physicians for veteran exams.</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
+          <t>‘Connect With a Recruiter’ form (veteranfeedback@vesservices.com = feedback only)</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>MO-licensed MD/DO; exams only, no treatment.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>MO examiner network.</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>Verify intake contact.</t>
+      <c r="L4" s="5" t="inlineStr">
+        <is>
+          <t>Verified provider page.</t>
         </is>
       </c>
     </row>
@@ -696,7 +728,7 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Optum Serve (formerly LHI / Logistics Health Inc)</t>
+          <t>Optum Serve (formerly LHI / Logistics Health)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -706,7 +738,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>VA &amp; federal medical exam contractor; disability + readiness exams.</t>
+          <t>VA &amp; federal medical disability/readiness exam contractor.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -716,27 +748,37 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>optumserve.com</t>
+          <t>providers.optumserve.com/recruitment/provider-form</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>'Providers' / network participation; credentialing via Optum.</t>
+          <t>Online form only</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
+          <t>Online form only</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>Complete the ‘Join the Network’ recruitment form; MO license required.</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
           <t>Active VA exam volume in MO.</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Verify provider onboarding path.</t>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Verified recruitment form URL.</t>
         </is>
       </c>
     </row>
@@ -766,27 +808,37 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>loyalsource.com</t>
+          <t>loyalsource.com/technical/mdeproviders</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Clinician opportunities / provider application.</t>
+          <t>Form (loyalsource.com/contact-us)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
+          <t>Web form only</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>MDE provider-partner inquiry form to perform VA C&amp;P exams at MO-area clinics.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
           <t>Places clinicians on MO-area contracts.</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="K6" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>Good secondary VA channel.</t>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Secondary VA channel.</t>
         </is>
       </c>
     </row>
@@ -806,7 +858,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Contracts physicians for VA and government medical evaluations.</t>
+          <t>Contracts physicians for VA and government medical evaluations (family practice listed).</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -816,27 +868,37 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>sterlingmedical.com</t>
+          <t>sterlingmedcorp.com/healthcare-provider-opportunities/physicians</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Provider / careers inquiry.</t>
+          <t>Web form</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
+          <t>Web form</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>Apply via Physicians opportunities page for VA-contract placements.</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
           <t>Recruits across states incl. MO.</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="K7" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>Verify if currently staffing MO.</t>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Correct domain: sterlingmedcorp.com (not sterlingmedical.com).</t>
         </is>
       </c>
     </row>
@@ -855,6 +917,8 @@
       <c r="H8" s="3" t="n"/>
       <c r="I8" s="3" t="n"/>
       <c r="J8" s="3" t="n"/>
+      <c r="K8" s="3" t="n"/>
+      <c r="L8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
@@ -867,7 +931,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>State SSA disability agency</t>
+          <t>State SSA disability agency (under DESE Voc Rehab)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -877,32 +941,42 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Disability consultative exams (adult/peds, mental, physical)</t>
+          <t>Disability consultative exams (physical &amp; mental)</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>dss.mo.gov (Family Support Division / DDS)</t>
+          <t>dese.mo.gov/adult-learning-rehabilitation-services/disability-determination</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Contact MO DDS Professional Relations Officer to become a CE provider.</t>
+          <t>573-290-5710 (PRO — verify)</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>THE primary in-state SSA disability channel.</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+          <t>Via PRO phone; SSA PRO locator: ssa.gov/disability/professionals/procontacts.htm</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>Contact the DDS Professional Relations Officer to enroll as a CE provider; MO license required.</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Primary in-state SSA disability channel.</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>Ask specifically about CE provider enrollment + fee schedule.</t>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Correction: MO DDS is under DESE (Voc Rehab), NOT DSS/Family Support Division.</t>
         </is>
       </c>
     </row>
@@ -912,17 +986,17 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>MDExams / MDSI (Medical Diagnostic Services)</t>
+          <t>MDSI – Medical Diagnostic Services Inc.</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>SSA CE scheduling vendor</t>
+          <t>SSA / disability eval vendor</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>National vendor that schedules SSA consultative exams into local clinics.</t>
+          <t>Contracts physicians as independent consultants for disability evaluations nationwide.</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -932,27 +1006,37 @@
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>mdexams.com</t>
+          <t>mdsiphysicians.com (‘Join Our Network’)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>'Become a provider' / clinic partnership inquiry.</t>
+          <t>800-548-9092 / 801-627-1093</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>Places SSA CE volume with MO clinics.</t>
-        </is>
-      </c>
-      <c r="I10" s="7" t="inlineStr">
+          <t>info@mdsiphysicians.com</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Contact corporate to join the consultant network.</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Places disability eval volume.</t>
+        </is>
+      </c>
+      <c r="K10" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>Verify MO coverage.</t>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>‘mdexams.com’ didn’t resolve — confirm MDSI is the vendor you meant.</t>
         </is>
       </c>
     </row>
@@ -982,25 +1066,35 @@
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>danestreet.com</t>
+          <t>site.danestreet.com/physician-network</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>'Join our panel' / physician panel application.</t>
+          <t>Request-info form</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
+          <t>marketing@danestreet.com</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Submit interest; panel admission after Credentialing Committee review (ABMS board cert).</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
           <t>Recruits MO examiners.</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="L11" s="5" t="inlineStr">
         <is>
           <t>Covers both IME and disability — strong fit.</t>
         </is>
@@ -1021,6 +1115,8 @@
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="3" t="n"/>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -1048,25 +1144,35 @@
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>examworks.com</t>
+          <t>examworks.com/physicians/medical-panel</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>'Join our panel of physicians' / provider recruitment.</t>
+          <t>206-200-7171 (recruiter — verify)</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Active MO case volume; needs local examiners.</t>
-        </is>
-      </c>
-      <c r="I13" s="6" t="inlineStr">
+          <t>Erica.seversen@examworks.com (verify)</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>Join medical panel; most states require ABMS/AOA board cert + ~8 hrs/wk patient care.</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>Active MO case volume.</t>
+        </is>
+      </c>
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="L13" s="5" t="inlineStr">
         <is>
           <t>Anchor IME target.</t>
         </is>
@@ -1098,25 +1204,35 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>mesgroup.com</t>
+          <t>messolutions.com/physician-consulting</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Provider / physician panel application.</t>
+          <t>Web form</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
+          <t>Web form</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Apply via Physician Consulting page; board-certified, active-practice.</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
           <t>Serves MO payers.</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="K14" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="L14" s="5" t="inlineStr">
         <is>
           <t>Same group as ExamWorks — one outreach may cover both.</t>
         </is>
@@ -1148,27 +1264,37 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>mcn.com</t>
+          <t>mcn.com/join</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>'Providers' &gt; join network.</t>
+          <t>Web form</t>
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
+          <t>ntamashiro@mcn.com (email CV)</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Email CV or use Join form; credentialing docs at mcn.com/providerdocs.</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
           <t>Recruits MO physicians.</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="K15" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>Verify MO need.</t>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Verified.</t>
         </is>
       </c>
     </row>
@@ -1198,25 +1324,35 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>genexservices.com</t>
+          <t>genexservices.com/solutions/clinical-services/ime/physician-panel</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Provider network inquiry.</t>
+          <t>Web form</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
+          <t>Web form</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Apply via IME Physician Panel page (URAC-credentialed).</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
           <t>MO workers' comp footprint.</t>
         </is>
       </c>
-      <c r="I16" s="7" t="inlineStr">
+      <c r="K16" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>Part of Enlyte/Mitchell.</t>
         </is>
@@ -1228,7 +1364,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>IMX Medical Management Services</t>
+          <t>IMX Medical Mgmt → Leidos QTC Health Services</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1238,7 +1374,7 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Independent medical exams and record reviews for insurers/attorneys.</t>
+          <t>Independent medical exams and record reviews (rebranded under Leidos QTC, Jan 2025).</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1248,27 +1384,37 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>imxmed.com</t>
+          <t>qtcm.com/imxmed/physician-panel</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Provider application.</t>
+          <t>Web form</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Places cases regionally incl. MO.</t>
-        </is>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
+          <t>Web form</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Apply via IMX Physician Panel page; board-certified physicians.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>Regional incl. MO.</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>Verify MO coverage.</t>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Now overlaps with #1 (QTC) — apply once.</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1434,7 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Workers' comp third-party administrator; uses IME/exam providers.</t>
+          <t>Workers' comp third-party administrator; uses IME/exam providers (PPO).</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1298,34 +1444,44 @@
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>corvel.com</t>
+          <t>corvel.com/provider-relations</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Provider / network inquiry.</t>
+          <t>Local CorVel rep</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
+          <t>Via Provider Relations page</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Download practitioner roster template, return to CorVel network contact; re-credential every 3 yrs.</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
           <t>TPA active in MO.</t>
         </is>
       </c>
-      <c r="I18" s="7" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>True 'TPA' in workers' comp sense.</t>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>True 'TPA' in the workers'-comp sense.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>Missouri state &amp; government bodies (direct credentialing / listings)</t>
+          <t>Missouri state &amp; government bodies (credentialing / listings / referral)</t>
         </is>
       </c>
       <c r="B19" s="3" t="n"/>
@@ -1337,6 +1493,8 @@
       <c r="H19" s="3" t="n"/>
       <c r="I19" s="3" t="n"/>
       <c r="J19" s="3" t="n"/>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
@@ -1344,7 +1502,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Missouri Division of Workers' Compensation (Dept. of Labor)</t>
+          <t>Missouri Division of Workers' Compensation (DOLIR)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -1354,7 +1512,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Administers MO workers' comp; independent medical exams &amp; ratings used in claims.</t>
+          <t>Administers MO workers' comp; physician IMEs (§287.140) &amp; disability ratings.</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1364,27 +1522,37 @@
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>labor.mo.gov/dwc</t>
+          <t>labor.mo.gov/dwc/healthcare-providers</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Review provider/exam requirements; get listed where applicable.</t>
+          <t>573-751-4231 / 800-775-2667</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
+          <t>workerscomp@labor.mo.gov</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Informational only — no network. Physician of claimant's choosing is permitted.</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
           <t>Statewide authority on MO workers' comp IMEs.</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>Understand MO rating rules (AMA Guides) before marketing.</t>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Use to understand MO rating rules (AMA Guides) before marketing — not an enrollment channel.</t>
         </is>
       </c>
     </row>
@@ -1414,27 +1582,37 @@
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>mvc.dps.mo.gov</t>
+          <t>mvc.dps.mo.gov/service (CVSO locator)</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Introduce GFM IME/Nexus services to MVC &amp; County Veterans Service Officers.</t>
+          <t>573-751-3779 HQ · 816-356-4075 KC</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
+          <t>mvc.dps.mo.gov/contact-us</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Use the Service Officer Locator to reach the nearest County Veterans Service Officer.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
           <t>Direct line to MO veterans needing evidence.</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr">
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>Referral relationship, not a TPA — high-value.</t>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>High-value referral relationship.</t>
         </is>
       </c>
     </row>
@@ -1453,6 +1631,8 @@
       <c r="H22" s="3" t="n"/>
       <c r="I22" s="3" t="n"/>
       <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n">
@@ -1460,7 +1640,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Missouri workers' comp &amp; personal-injury attorneys</t>
+          <t>Missouri workers'-comp &amp; personal-injury attorneys</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1480,27 +1660,37 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>Local firms (e.g., Boyd, Kenter, Thomas &amp; Parrish – already in your files)</t>
+          <t>Firm sites (e.g., Boyd, Kenter, Thomas &amp; Parrish — already in your files)</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Targeted outreach with fee schedule + turnaround (you already emailed BKTP).</t>
+          <t>Per firm</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
+          <t>Per firm</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Targeted outreach with fee schedule + work sample; you already emailed BKTP.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
           <t>Local Jackson County / KC metro firms.</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr">
+      <c r="K23" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>Warm channel — you already have an IME report for a BKTP case (M. Mendez).</t>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Warm channel — you delivered the M. Mendez IME for BKTP.</t>
         </is>
       </c>
     </row>
@@ -1530,27 +1720,37 @@
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>matalaw.com</t>
+          <t>matanet.org (advertising/sponsorship)</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Sponsor / directory listing / educational outreach.</t>
+          <t>Site contact</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
+          <t>Contact form</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Sponsor / advertise to reach the plaintiff bar; no public expert directory.</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
           <t>Statewide plaintiff attorney audience.</t>
         </is>
       </c>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="K24" s="7" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>Marketing channel to many firms at once.</t>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>Correct domain: matanet.org (not matalaw.com).</t>
         </is>
       </c>
     </row>
@@ -1560,7 +1760,7 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>DAV / VFW / American Legion (Missouri departments)</t>
+          <t>DAV · VFW · American Legion (Missouri departments)</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
@@ -1580,27 +1780,37 @@
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>dav.org · vfwmo.org · molegion.org</t>
+          <t>DAV: davwebsites.dav.org/mo · VFW: vfwmo.org/veteran-service-officer-resources · Legion: missourilegion.org/contact-us</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
+          <t>DAV KC 816-765-8787 · VFW HQ 573-636-8761 · Legion Svc 573-761-4143</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>services@missourilegion.org (Legion); DAV/VFW via forms</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
           <t>Introduce Veterans@Work IME + Nexus services to MO service officers.</t>
         </is>
       </c>
-      <c r="H25" s="5" t="inlineStr">
+      <c r="J25" s="5" t="inlineStr">
         <is>
           <t>Large MO veteran membership.</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr">
+      <c r="K25" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>Pairs with Missouri Veterans Commission outreach.</t>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Legion domain is missourilegion.org.</t>
         </is>
       </c>
     </row>
@@ -1610,7 +1820,7 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>County Veterans Service Officers (Jackson, Clay, Cass, etc.)</t>
+          <t>County Veterans Service Officers (Jackson, Cass, etc.)</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -1630,25 +1840,35 @@
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>County govt veteran services pages</t>
+          <t>jacksongov.org/Residents/Health-Services/Veteran-BenefitsServices</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Direct relationship-building with local CVSOs.</t>
+          <t>816-325-5883 / 816-325-5882</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
+          <t>Call office</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Independence office (Mon–Fri 8–4) serves Jackson &amp; Cass Counties.</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
           <t>Local, high-trust referrals.</t>
         </is>
       </c>
-      <c r="I26" s="6" t="inlineStr">
+      <c r="K26" s="6" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="J26" s="5" t="inlineStr">
+      <c r="L26" s="5" t="inlineStr">
         <is>
           <t>Start with your home counties.</t>
         </is>
@@ -1656,11 +1876,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A8:J8"/>
-    <mergeCell ref="A22:J22"/>
-    <mergeCell ref="A12:J12"/>
-    <mergeCell ref="A2:J2"/>
-    <mergeCell ref="A19:J19"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A19:L19"/>
+    <mergeCell ref="A8:L8"/>
+    <mergeCell ref="A22:L22"/>
+    <mergeCell ref="A12:L12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1672,11 +1892,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="95" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1685,133 +1905,129 @@
           <t>Garcia Family Medicine — Missouri Disability &amp; IME Outreach List</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr"/>
+      <c r="B1" t="inlineStr"/>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr"/>
-      <c r="B2" s="10" t="inlineStr"/>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Contacts researched / verified</t>
+        </is>
+      </c>
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-02. Websites are official domains; most networks funnel applicants through web forms, so exact recruiter emails/phones are often not published. Items marked 'verify' should be confirmed on the live page before use. No phone/email was invented.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Purpose</t>
-        </is>
-      </c>
-      <c r="B3" s="10" t="inlineStr">
-        <is>
-          <t>Organizations to approach so GFM (Dr. Tess) receives a steady flow of disability and IME work: VA disability (C&amp;P) exams, Social Security consultative exams, and workers'-comp/auto/legal IMEs.</t>
-        </is>
-      </c>
+      <c r="A3" s="12" t="inlineStr"/>
+      <c r="B3" s="11" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="11" t="inlineStr"/>
-      <c r="B4" s="10" t="inlineStr"/>
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Three ways the work flows in</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Three ways the work flows in</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="inlineStr"/>
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>1. VA disability TPAs</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>QTC, VES, Optum Serve, Loyal Source, Sterling credential you as a network examiner for veteran C&amp;P disability exams. Highest volume.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>1. VA disability TPAs</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="inlineStr">
-        <is>
-          <t>QTC, VES, Optum Serve, etc. contract you as a network examiner to perform veteran C&amp;P disability exams. Highest volume; requires credentialing.</t>
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>2. SSA disability (CE)</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Missouri DDS (under DESE Voc Rehab) pays providers for Consultative Exams. MDSI / Dane Street also place disability evals.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>2. SSA disability (CE)</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="inlineStr">
-        <is>
-          <t>Missouri DDS pays providers to examine Social Security claimants (Consultative Exams). MDExams/Dane Street also schedule these into clinics.</t>
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>3. IME networks &amp; attorneys</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>ExamWorks, Dane Street, MCN, Genex, CorVel place workers'-comp/auto/legal IMEs. Attorneys &amp; VSOs send claimants directly for IMEs and nexus letters.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>3. IME networks &amp; attorneys</t>
-        </is>
-      </c>
-      <c r="B8" s="10" t="inlineStr">
-        <is>
-          <t>ExamWorks, Dane Street, MCN, etc. place workers'-comp/auto/legal IME cases. Attorneys &amp; VSOs send claimants directly for IMEs and nexus letters.</t>
-        </is>
-      </c>
+      <c r="A8" s="12" t="inlineStr"/>
+      <c r="B8" s="11" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Priority key</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>HIGH = start here (volume or warm relationship). MED = solid secondary. LOW = verify fit / informational only.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Priority key</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>HIGH = start here (volume or warm relationship). MED = solid secondary. LOW = verify fit first.</t>
-        </is>
-      </c>
+      <c r="A10" s="12" t="inlineStr"/>
+      <c r="B10" s="11" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr"/>
-      <c r="B11" s="10" t="inlineStr"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Corrections from research</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>• MO DDS is under DESE (Voc Rehab), not DSS/FSD.  • IMX is now Leidos QTC (overlaps #1).  • MATA domain is matanet.org.  • American Legion MO is missourilegion.org.  • Sterling is sterlingmedcorp.com.  • 'mdexams.com' → MDSI (mdsiphysicians.com) — confirm intended vendor.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr"/>
+      <c r="B12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>Suggested first moves</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>1) Apply to QTC + VES + Optum Serve (VA). 2) Call Missouri DDS about CE provider enrollment. 3) Join ExamWorks + Dane Street panels. 4) Re-contact BKTP and pitch CVSOs/DAV with your Veterans@Work IME + Nexus packet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="inlineStr"/>
-      <c r="B13" s="10" t="inlineStr"/>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>1) Apply to QTC + VES + Optum Serve (VA). 2) Call Missouri DDS PRO about CE enrollment. 3) Join ExamWorks + Dane Street panels. 4) Re-contact BKTP and pitch CVSOs/DAV/VFW/Legion with the Veterans@Work IME + Nexus packet.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>IMPORTANT — verify before sending</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Websites listed are the official company domains, but exact provider-intake emails/phone numbers change. Confirm the current 'join our network / become a provider' contact on each site before applying. Do not treat any contact detail here as final.</t>
-        </is>
-      </c>
+      <c r="A14" s="12" t="inlineStr"/>
+      <c r="B14" s="11" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr"/>
-      <c r="B15" s="10" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Assets you already have to attach</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>• IME service + pricing sheet  • Veterans@Work IME Referral Flyer + sample MoU  • Nexus Letter Services doc  • A completed IME report (M. Mendez) as a work sample.</t>
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Assets to attach</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>• IME service + pricing sheet  • Veterans@Work IME Referral Flyer + sample MoU  • Nexus Letter Services doc  • completed IME report (M. Mendez) as a work sample.  • The outreach packet (5 email templates) accompanies this list.</t>
         </is>
       </c>
     </row>

</xml_diff>